<commit_message>
data: data entry for mar 19 2026 completed
</commit_message>
<xml_diff>
--- a/data/daily_metrics.xlsx
+++ b/data/daily_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3841b178c28d2367/Documents/GitHub/marketing-impact-lab/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E889DAE2-D19B-423B-8702-66CCA2A5F95F}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F70FC03-74A7-45A3-95FF-31E1009A4F92}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD93D2A4-EDB6-4118-BB9A-85CF088B22DB}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>date</t>
   </si>
@@ -608,6 +608,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -927,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B109BE1C-3681-4489-A773-FCDC5502B018}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1013,6 +1017,41 @@
         <v>17</v>
       </c>
     </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46100</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data:entry for 3-20-2026 completed
</commit_message>
<xml_diff>
--- a/data/daily_metrics.xlsx
+++ b/data/daily_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3841b178c28d2367/Documents/GitHub/marketing-impact-lab/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F70FC03-74A7-45A3-95FF-31E1009A4F92}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEAADAB6-19A8-421E-A885-3B33EA83A32C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD93D2A4-EDB6-4118-BB9A-85CF088B22DB}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
   <si>
     <t>date</t>
   </si>
@@ -931,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B109BE1C-3681-4489-A773-FCDC5502B018}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1052,6 +1052,41 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
img: ga4 ss 3-21-26
</commit_message>
<xml_diff>
--- a/data/daily_metrics.xlsx
+++ b/data/daily_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3841b178c28d2367/Documents/GitHub/marketing-impact-lab/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEAADAB6-19A8-421E-A885-3B33EA83A32C}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F50F270-693C-4F7A-97CE-E708674E444F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD93D2A4-EDB6-4118-BB9A-85CF088B22DB}"/>
+    <workbookView xWindow="4380" yWindow="195" windowWidth="21600" windowHeight="11295" xr2:uid="{BD93D2A4-EDB6-4118-BB9A-85CF088B22DB}"/>
   </bookViews>
   <sheets>
     <sheet name="daily_metrics" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
   <si>
     <t>date</t>
   </si>
@@ -931,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B109BE1C-3681-4489-A773-FCDC5502B018}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1087,6 +1087,41 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>46102</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
img:screenshots and data collected for 3/22 and 3/23
</commit_message>
<xml_diff>
--- a/data/daily_metrics.xlsx
+++ b/data/daily_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3841b178c28d2367/Documents/GitHub/marketing-impact-lab/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F50F270-693C-4F7A-97CE-E708674E444F}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{76A1B050-581A-48A7-8802-028AEC8AE983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{037DBDA5-2593-4581-B6EC-015EB8B99D7D}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="195" windowWidth="21600" windowHeight="11295" xr2:uid="{BD93D2A4-EDB6-4118-BB9A-85CF088B22DB}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="16">
   <si>
     <t>date</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t>project_click</t>
+  </si>
+  <si>
+    <t>linkedin test</t>
   </si>
 </sst>
 </file>
@@ -931,7 +934,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B109BE1C-3681-4489-A773-FCDC5502B018}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1122,6 +1125,76 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>46103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46076</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>